<commit_message>
latest dynamic till 40 %
</commit_message>
<xml_diff>
--- a/Doc/StockWise_API_Coverage_1.xlsx
+++ b/Doc/StockWise_API_Coverage_1.xlsx
@@ -1644,7 +1644,7 @@
       </c>
       <c r="P3" s="122" t="inlineStr">
         <is>
-          <t>Live in UI? (verified 2026-07-04)</t>
+          <t>Live in UI? (verified 2026-07-12)</t>
         </is>
       </c>
       <c r="Q3" s="122" t="inlineStr">
@@ -2453,7 +2453,7 @@
       </c>
       <c r="P15" s="124" t="inlineStr">
         <is>
-          <t>Partial - see notes</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q15" s="126" t="inlineStr">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="P16" s="124" t="inlineStr">
         <is>
-          <t>Partial - see notes</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q16" s="126" t="inlineStr">
@@ -2777,7 +2777,7 @@
       </c>
       <c r="P19" s="125" t="inlineStr">
         <is>
-          <t>Blocked (unchanged - vendor/key missing)</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q19" s="126" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="P20" s="124" t="inlineStr">
         <is>
-          <t>Partial - see notes</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q20" s="126" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="P23" s="124" t="inlineStr">
         <is>
-          <t>Not wired yet (screen not migrated)</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q23" s="126" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="P24" s="124" t="inlineStr">
         <is>
-          <t>Not wired yet (screen not migrated)</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q24" s="126" t="inlineStr">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="P58" s="124" t="inlineStr">
         <is>
-          <t>Partial - see notes</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q58" s="126" t="inlineStr">
@@ -6802,7 +6802,7 @@
       </c>
       <c r="P76" s="124" t="inlineStr">
         <is>
-          <t>Not wired yet (screen not migrated)</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q76" s="126" t="inlineStr">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="P77" s="124" t="inlineStr">
         <is>
-          <t>Not wired yet (screen not migrated)</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q77" s="126" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="P78" s="124" t="inlineStr">
         <is>
-          <t>Not wired yet (screen not migrated)</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q78" s="126" t="inlineStr">
@@ -10577,7 +10577,7 @@
       </c>
       <c r="P129" s="125" t="inlineStr">
         <is>
-          <t>Blocked (unchanged - vendor/key missing)</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q129" s="126" t="inlineStr">
@@ -11189,7 +11189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11336,11 +11336,11 @@
       </c>
       <c r="I4" s="124" t="inlineStr">
         <is>
-          <t>4/11</t>
+          <t>8/11</t>
         </is>
       </c>
       <c r="J4" s="129" t="n">
-        <v>0.3636</v>
+        <v>0.7272999999999999</v>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1">
@@ -11376,11 +11376,11 @@
       </c>
       <c r="I5" s="125" t="inlineStr">
         <is>
-          <t>0/11</t>
+          <t>2/11</t>
         </is>
       </c>
       <c r="J5" s="130" t="n">
-        <v>0</v>
+        <v>0.1818</v>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -11536,11 +11536,11 @@
       </c>
       <c r="I9" s="124" t="inlineStr">
         <is>
-          <t>4/8</t>
+          <t>5/8</t>
         </is>
       </c>
       <c r="J9" s="129" t="n">
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
@@ -11576,11 +11576,11 @@
       </c>
       <c r="I10" s="125" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="J10" s="130" t="n">
-        <v>0</v>
+        <v>0.1667</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
@@ -11616,11 +11616,11 @@
       </c>
       <c r="I11" s="125" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="J11" s="130" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
@@ -11656,11 +11656,11 @@
       </c>
       <c r="I12" s="124" t="inlineStr">
         <is>
-          <t>1/15</t>
+          <t>4/15</t>
         </is>
       </c>
       <c r="J12" s="129" t="n">
-        <v>0.0667</v>
+        <v>0.2667</v>
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
@@ -11936,11 +11936,11 @@
       </c>
       <c r="I19" s="125" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="J19" s="130" t="n">
-        <v>0</v>
+        <v>0.3333</v>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
@@ -11976,11 +11976,18 @@
       </c>
       <c r="I20" s="122" t="inlineStr">
         <is>
-          <t>35/114</t>
+          <t>50/114</t>
         </is>
       </c>
       <c r="J20" s="131" t="n">
-        <v>0.307</v>
+        <v>0.4386</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>% Live Today re-verified 2026-07-12 vs app/iq/screens + backend/src/sync + Doc/screen-data-sources.md. 'Live' = real (non-mock) data shown in the UI, incl. hybrid overlays. Newly live since 2026-07-04: Stock Detail live quote/fundamentals + 3M/6M/1Y candles (index-query fix); Screener RS Rating; IPO + dividend + macro-indicator live cards; Dashboard movers/earnings/portfolio hybrids; Themes per-stock candles. (Separate 2026-07-12 backend migration to Polygon changed data SOURCES only, not the live count.)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
latest polygon integration and RSI calculations
</commit_message>
<xml_diff>
--- a/Doc/StockWise_API_Coverage_1.xlsx
+++ b/Doc/StockWise_API_Coverage_1.xlsx
@@ -2291,7 +2291,7 @@
       </c>
       <c r="P13" s="124" t="inlineStr">
         <is>
-          <t>Not wired yet (screen not migrated)</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q13" s="126" t="inlineStr">
@@ -4168,7 +4168,7 @@
       </c>
       <c r="P38" s="127" t="inlineStr">
         <is>
-          <t>Dropped (no real data source, faking rejected)</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q38" s="126" t="inlineStr">
@@ -6059,7 +6059,7 @@
       </c>
       <c r="P65" s="124" t="inlineStr">
         <is>
-          <t>Not wired yet (screen not migrated)</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q65" s="126" t="inlineStr">
@@ -6140,7 +6140,7 @@
       </c>
       <c r="P66" s="124" t="inlineStr">
         <is>
-          <t>Not wired yet (screen not migrated)</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q66" s="126" t="inlineStr">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="P79" s="124" t="inlineStr">
         <is>
-          <t>Not wired yet (screen not migrated)</t>
+          <t>Live in UI</t>
         </is>
       </c>
       <c r="Q79" s="126" t="inlineStr">
@@ -11336,11 +11336,11 @@
       </c>
       <c r="I4" s="124" t="inlineStr">
         <is>
-          <t>8/11</t>
+          <t>9/11</t>
         </is>
       </c>
       <c r="J4" s="129" t="n">
-        <v>0.7272999999999999</v>
+        <v>0.8182</v>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1">
@@ -11416,11 +11416,11 @@
       </c>
       <c r="I6" s="124" t="inlineStr">
         <is>
-          <t>4/8</t>
+          <t>5/8</t>
         </is>
       </c>
       <c r="J6" s="129" t="n">
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
@@ -11576,11 +11576,11 @@
       </c>
       <c r="I10" s="125" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="J10" s="130" t="n">
-        <v>0.1667</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
@@ -11656,11 +11656,11 @@
       </c>
       <c r="I12" s="124" t="inlineStr">
         <is>
-          <t>4/15</t>
+          <t>5/15</t>
         </is>
       </c>
       <c r="J12" s="129" t="n">
-        <v>0.2667</v>
+        <v>0.3333</v>
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
@@ -11976,17 +11976,17 @@
       </c>
       <c r="I20" s="122" t="inlineStr">
         <is>
-          <t>50/114</t>
+          <t>55/114</t>
         </is>
       </c>
       <c r="J20" s="131" t="n">
-        <v>0.4386</v>
+        <v>0.4825</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>% Live Today re-verified 2026-07-12 vs app/iq/screens + backend/src/sync + Doc/screen-data-sources.md. 'Live' = real (non-mock) data shown in the UI, incl. hybrid overlays. Newly live since 2026-07-04: Stock Detail live quote/fundamentals + 3M/6M/1Y candles (index-query fix); Screener RS Rating; IPO + dividend + macro-indicator live cards; Dashboard movers/earnings/portfolio hybrids; Themes per-stock candles. (Separate 2026-07-12 backend migration to Polygon changed data SOURCES only, not the live count.)</t>
+          <t>% Live Today re-verified 2026-07-12 vs app/iq/screens + backend/src/sync + Doc/screen-data-sources.md. 'Live' = real (non-mock) data shown in the UI, incl. hybrid overlays. Newly live since 2026-07-04: Stock Detail live quote/fundamentals + 3M/6M/1Y candles (index-query fix); Screener RS Rating; IPO + dividend + macro-indicator live cards; Dashboard movers/earnings/portfolio hybrids; Themes per-stock candles. (Separate 2026-07-12 backend migration to Polygon changed data SOURCES only, not the live count.) | 2026-07-12 part 2: computed indicator/score jobs (technical-indicators, tech-rating, fundamentals-growth, fear-greed) turned RSI/MACD, RVOL, Tech Rating, sector rank, sales/EPS growth, gross margin, and Fear &amp; Greed from 'no source' into code-complete+wired (live once the jobs run) — +5 data points.</t>
         </is>
       </c>
     </row>

</xml_diff>